<commit_message>
section under video 4
Automated migration updates generated by Experience Modernization Agent.

Changed files (12):
- blocks/service-panels/_service-panels.json
- blocks/service-panels/metadata.json
- blocks/service-panels/service-panels.css
- blocks/service-panels/service-panels.js
- component-definition.json
- component-filters.json
- tools/importer/import-home.bundle.js
- tools/importer/import-home.js
- tools/importer/page-templates.json
- tools/importer/parsers/service-panels.js
- tools/importer/reports/en-us.report.json
- tools/importer/reports/import-home.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -40,7 +40,7 @@
     <t>en-us.report.json</t>
   </si>
   <si>
-    <t>["hero-home","service-areas","marquee","cards-case-study","cards-case-study","cards-case-study","cards-partner","cards-industry","cards-insight","hero-cta"]</t>
+    <t>["hero-home","service-panels","marquee","cards-case-study","cards-case-study","cards-case-study","cards-partner","cards-industry","cards-insight","hero-cta"]</t>
   </si>
   <si>
     <t>en-us</t>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-02T07:08:34.542Z</t>
+    <t>2026-09-02T09:31:17.507Z</t>
   </si>
   <si>
     <t>Home | Credera</t>

</xml_diff>

<commit_message>
migration for home template pages
Automated migration updates generated by Experience Modernization Agent.

Changed files (6):
- tools/importer/reports/en-us.report.json
- tools/importer/reports/en-us/contact/forrester-wave-marketing-creative-and-content-services-q1-2025.report.json
- tools/importer/reports/en-us/europe-asia-pacific-privacy-notice.report.json
- tools/importer/reports/en-us/insights/credera-s-mobile-expert-to-speak-at-the-7th-annual-demogala-showcase-and-innovation-conference.report.json
- tools/importer/reports/en-us/insights/what-s-happening-with-your-business-the-twitter-e-commerce-partnership.report.json
- tools/importer/reports/import-home.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,13 +52,67 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-02T18:48:20.977Z</t>
+    <t>2026-09-07T19:24:14.437Z</t>
   </si>
   <si>
     <t>Home | Credera</t>
   </si>
   <si>
     <t>https://credera.com/en-us</t>
+  </si>
+  <si>
+    <t>en-us/europe-asia-pacific-privacy-notice.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>en-us/europe-asia-pacific-privacy-notice</t>
+  </si>
+  <si>
+    <t>2026-09-07T19:24:26.153Z</t>
+  </si>
+  <si>
+    <t>Europe | Asia-Pacific Privacy Notice | Credera</t>
+  </si>
+  <si>
+    <t>https://credera.com/en-us/europe-asia-pacific-privacy-notice</t>
+  </si>
+  <si>
+    <t>en-us/contact/forrester-wave-marketing-creative-and-content-services-q1-2025.report.json</t>
+  </si>
+  <si>
+    <t>en-us/contact/forrester-wave-marketing-creative-and-content-services-q1-2025</t>
+  </si>
+  <si>
+    <t>2026-09-07T19:24:20.195Z</t>
+  </si>
+  <si>
+    <t>https://credera.com/en-us/contact/forrester-wave-marketing-creative-and-content-services-q1-2025</t>
+  </si>
+  <si>
+    <t>en-us/insights/credera-s-mobile-expert-to-speak-at-the-7th-annual-demogala-showcase-and-innovation-conference.report.json</t>
+  </si>
+  <si>
+    <t>en-us/insights/credera-s-mobile-expert-to-speak-at-the-7th-annual-demogala-showcase-and-innovation-conference</t>
+  </si>
+  <si>
+    <t>2026-09-07T19:24:38.339Z</t>
+  </si>
+  <si>
+    <t>https://credera.com/en-us/insights/credera%e2%80%99s-mobile-expert-to-speak-at-the-7th-annual-demogala-showcase-and-innovation-conference</t>
+  </si>
+  <si>
+    <t>en-us/insights/what-s-happening-with-your-business-the-twitter-e-commerce-partnership.report.json</t>
+  </si>
+  <si>
+    <t>en-us/insights/what-s-happening-with-your-business-the-twitter-e-commerce-partnership</t>
+  </si>
+  <si>
+    <t>2026-09-07T19:24:32.195Z</t>
+  </si>
+  <si>
+    <t>https://credera.com/en-us/insights/%e2%80%9cwhat%e2%80%99s-happening%e2%80%9d-with-your-business-the-twitter-e-commerce-partnership</t>
   </si>
 </sst>
 </file>
@@ -447,16 +501,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="27" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +561,110 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>